<commit_message>
docs: move charge attack review to a separate hold sheet
</commit_message>
<xml_diff>
--- a/outputs/01a151d0-9d92-7900-b5be-31a811469c9d/풀로세움_효과와스킬_분류_v3.xlsx
+++ b/outputs/01a151d0-9d92-7900-b5be-31a811469c9d/풀로세움_효과와스킬_분류_v3.xlsx
@@ -17,6 +17,7 @@
     <sheet name="스킬 분류" sheetId="2" r:id="rId2"/>
     <sheet name="검토 대기" sheetId="3" r:id="rId3"/>
     <sheet name="미분류·잔여" sheetId="4" r:id="rId4"/>
+    <sheet name="보류" sheetId="5" r:id="rId8"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -4732,7 +4733,7 @@
   <sheetPr>
     <tabColor rgb="FFB58B37"/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -4886,331 +4887,345 @@
     <row r="10" spans="1:7" ht="42" customHeight="1">
       <c r="A10" s="47"/>
       <c r="B10" s="7" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>336</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="G10" s="28"/>
     </row>
     <row r="11" spans="1:7" ht="42" customHeight="1">
       <c r="A11" s="47"/>
       <c r="B11" s="7" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>336</v>
+        <v>345</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="G11" s="28"/>
     </row>
-    <row r="12" spans="1:7" ht="42" customHeight="1">
-      <c r="A12" s="47"/>
-      <c r="B12" s="7" t="s">
-        <v>342</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>343</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>344</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>345</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>346</v>
-      </c>
-      <c r="G12" s="28"/>
+    <row r="12" spans="1:7" ht="34" customHeight="1">
+      <c r="A12" s="48" t="s">
+        <v>347</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>348</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>349</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>350</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>351</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>352</v>
+      </c>
+      <c r="G12" s="27"/>
     </row>
     <row r="13" spans="1:7" ht="34" customHeight="1">
-      <c r="A13" s="48" t="s">
-        <v>347</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>348</v>
-      </c>
-      <c r="C13" s="11" t="s">
-        <v>349</v>
-      </c>
-      <c r="D13" s="9" t="s">
-        <v>350</v>
-      </c>
-      <c r="E13" s="9" t="s">
+      <c r="A13" s="49"/>
+      <c r="B13" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>354</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="F13" s="9" t="s">
-        <v>352</v>
-      </c>
-      <c r="G13" s="27"/>
-    </row>
-    <row r="14" spans="1:7" ht="34" customHeight="1">
+      <c r="F13" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="G13" s="28"/>
+    </row>
+    <row r="14" spans="1:7" ht="42" customHeight="1">
       <c r="A14" s="49"/>
       <c r="B14" s="10" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>351</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="G14" s="28"/>
     </row>
     <row r="15" spans="1:7" ht="42" customHeight="1">
       <c r="A15" s="49"/>
       <c r="B15" s="10" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>351</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="G15" s="28"/>
     </row>
     <row r="16" spans="1:7" ht="42" customHeight="1">
-      <c r="A16" s="49"/>
-      <c r="B16" s="10" t="s">
-        <v>361</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>362</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>363</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>351</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>364</v>
-      </c>
-      <c r="G16" s="28"/>
+      <c r="A16" s="50" t="s">
+        <v>365</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>366</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>367</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>368</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>369</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>370</v>
+      </c>
+      <c r="G16" s="27"/>
     </row>
     <row r="17" spans="1:7" ht="42" customHeight="1">
-      <c r="A17" s="50" t="s">
-        <v>365</v>
-      </c>
-      <c r="B17" s="13" t="s">
-        <v>366</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>367</v>
-      </c>
-      <c r="D17" s="9" t="s">
-        <v>368</v>
-      </c>
-      <c r="E17" s="9" t="s">
-        <v>369</v>
-      </c>
-      <c r="F17" s="9" t="s">
-        <v>370</v>
-      </c>
-      <c r="G17" s="27"/>
-    </row>
-    <row r="18" spans="1:7" ht="42" customHeight="1">
+      <c r="A17" s="51"/>
+      <c r="B17" s="12" t="s">
+        <v>371</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>372</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="G17" s="28"/>
+    </row>
+    <row r="18" spans="1:7" ht="34" customHeight="1">
       <c r="A18" s="51"/>
       <c r="B18" s="12" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>374</v>
+        <v>131</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="G18" s="28"/>
     </row>
     <row r="19" spans="1:7" ht="34" customHeight="1">
       <c r="A19" s="51"/>
       <c r="B19" s="12" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>131</v>
+        <v>225</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>379</v>
-      </c>
-      <c r="G19" s="28"/>
-    </row>
-    <row r="20" spans="1:7" ht="34" customHeight="1">
+        <v>383</v>
+      </c>
+      <c r="G19" s="28" t="inlineStr">
+        <is>
+          <t>능력치 버프·디버프의 정화 여부와 분리한다. 능력치 디버프는 정화 불가이며 상태이상 중첩 제거 범위만 미결.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="42" customHeight="1">
       <c r="A20" s="51"/>
       <c r="B20" s="12" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>382</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>225</v>
+        <v>386</v>
+      </c>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t>이로운 1턴 소분류(명칭 미정)</t>
+        </is>
       </c>
       <c r="F20" s="1" t="s">
-        <v>383</v>
-      </c>
-      <c r="G20" s="28" t="inlineStr">
-        <is>
-          <t>능력치 버프·디버프의 정화 여부와 분리한다. 능력치 디버프는 정화 불가이며 상태이상 중첩 제거 범위만 미결.</t>
-        </is>
-      </c>
+        <v>388</v>
+      </c>
+      <c r="G20" s="28"/>
     </row>
     <row r="21" spans="1:7" ht="42" customHeight="1">
       <c r="A21" s="51"/>
       <c r="B21" s="12" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>386</v>
-      </c>
-      <c r="E21" s="1" t="inlineStr">
-        <is>
-          <t>이로운 1턴 소분류(명칭 미정)</t>
-        </is>
+        <v>391</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>184</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>388</v>
-      </c>
-      <c r="G21" s="28"/>
+        <v>392</v>
+      </c>
+      <c r="G21" s="28" t="inlineStr">
+        <is>
+          <t>능력치 디버프는 정화 불가. 상대 정화 시 반환하는 기존 전제는 적용하지 않으며 다른 해제 연동은 미결.</t>
+        </is>
+      </c>
     </row>
     <row r="22" spans="1:7" ht="42" customHeight="1">
       <c r="A22" s="51"/>
       <c r="B22" s="12" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>184</v>
+        <v>396</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>392</v>
-      </c>
-      <c r="G22" s="28" t="inlineStr">
-        <is>
-          <t>능력치 디버프는 정화 불가. 상대 정화 시 반환하는 기존 전제는 적용하지 않으며 다른 해제 연동은 미결.</t>
-        </is>
-      </c>
+        <v>397</v>
+      </c>
+      <c r="G22" s="28"/>
     </row>
     <row r="23" spans="1:7" ht="42" customHeight="1">
       <c r="A23" s="51"/>
       <c r="B23" s="12" t="s">
-        <v>393</v>
+        <v>398</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>396</v>
+        <v>5</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="G23" s="28"/>
     </row>
-    <row r="24" spans="1:7" ht="42" customHeight="1">
-      <c r="A24" s="51"/>
-      <c r="B24" s="12" t="s">
-        <v>398</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>399</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>400</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="G24" s="28"/>
+    <row r="24" spans="1:7" ht="100" customHeight="1">
+      <c r="A24" s="51" t="inlineStr">
+        <is>
+          <t>추가 논의</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>1턴 소분류 이름</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>해로운 상태는 봉인·속박·도발·암실, 이로운 상태는 면역이다.</t>
+        </is>
+      </c>
+      <c r="D24" s="1" t="inlineStr">
+        <is>
+          <t>봉인·속박·도발·암실 / 면역</t>
+        </is>
+      </c>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t>명칭 미정(1턴)</t>
+        </is>
+      </c>
+      <c r="F24" s="1" t="inlineStr">
+        <is>
+          <t>해로운 쪽과 이로운 쪽의 소분류 이름</t>
+        </is>
+      </c>
+      <c r="G24" s="28" t="inlineStr">
+        <is>
+          <t>미결</t>
+        </is>
+      </c>
     </row>
     <row r="25" spans="1:7" ht="100" customHeight="1">
-      <c r="A25" s="51" t="inlineStr">
-        <is>
-          <t>추가 논의</t>
-        </is>
-      </c>
+      <c r="A25" s="51"/>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>1턴 소분류 이름</t>
+          <t>1턴의 시작과 종료</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>해로운 상태는 봉인·속박·도발·암실, 이로운 상태는 면역이다.</t>
+          <t>1턴만 부여한다는 기간은 확정, 부여 시점에 따른 종료 기준은 미정이다.</t>
         </is>
       </c>
       <c r="D25" s="1" t="inlineStr">
         <is>
-          <t>봉인·속박·도발·암실 / 면역</t>
+          <t>선공·후공 사용, 턴 끝의 포자 발동</t>
         </is>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>명칭 미정(1턴)</t>
+          <t>상태이상 공통 규칙</t>
         </is>
       </c>
       <c r="F25" s="1" t="inlineStr">
         <is>
-          <t>해로운 쪽과 이로운 쪽의 소분류 이름</t>
+          <t>이번 턴 종료인지 다음 해당 행동까지인지</t>
         </is>
       </c>
       <c r="G25" s="28" t="inlineStr">
@@ -5223,27 +5238,27 @@
       <c r="A26" s="51"/>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>1턴의 시작과 종료</t>
+          <t>속박 스킬 허용</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>1턴만 부여한다는 기간은 확정, 부여 시점에 따른 종료 기준은 미정이다.</t>
+          <t>속박만 있는 스킬은 두지 않고 항상 부가 상태이상으로 연결한다.</t>
         </is>
       </c>
       <c r="D26" s="1" t="inlineStr">
         <is>
-          <t>선공·후공 사용, 턴 끝의 포자 발동</t>
+          <t>교체 제한 1턴</t>
         </is>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>상태이상 공통 규칙</t>
+          <t>해로운 1턴 상태</t>
         </is>
       </c>
       <c r="F26" s="1" t="inlineStr">
         <is>
-          <t>이번 턴 종료인지 다음 해당 행동까지인지</t>
+          <t>해당 기술을 허용할지, 어떤 부가 상태와 연결할지</t>
         </is>
       </c>
       <c r="G26" s="28" t="inlineStr">
@@ -5256,17 +5271,17 @@
       <c r="A27" s="51"/>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>속박 스킬 허용</t>
+          <t>속박 재부여·1:1</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>속박만 있는 스킬은 두지 않고 항상 부가 상태이상으로 연결한다.</t>
+          <t>한 식물에게 여러 번 사용 금지, 교체 시 초기화.</t>
         </is>
       </c>
       <c r="D27" s="1" t="inlineStr">
         <is>
-          <t>교체 제한 1턴</t>
+          <t>속박. 1:1에서 봉인처럼 취급할지 논의</t>
         </is>
       </c>
       <c r="E27" s="1" t="inlineStr">
@@ -5276,7 +5291,7 @@
       </c>
       <c r="F27" s="1" t="inlineStr">
         <is>
-          <t>해당 기술을 허용할지, 어떤 부가 상태와 연결할지</t>
+          <t>재사용 금지 범위·초기화 기준·1:1 처리</t>
         </is>
       </c>
       <c r="G27" s="28" t="inlineStr">
@@ -5289,17 +5304,17 @@
       <c r="A28" s="51"/>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>속박 재부여·1:1</t>
+          <t>도발과 복합 스킬</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>한 식물에게 여러 번 사용 금지, 교체 시 초기화.</t>
+          <t>방어스킬을 전부 제한한다는 사용자 편집을 유지한다.</t>
         </is>
       </c>
       <c r="D28" s="1" t="inlineStr">
         <is>
-          <t>속박. 1:1에서 봉인처럼 취급할지 논의</t>
+          <t>방어+공격·방어+다른 효과 스킬</t>
         </is>
       </c>
       <c r="E28" s="1" t="inlineStr">
@@ -5309,7 +5324,7 @@
       </c>
       <c r="F28" s="1" t="inlineStr">
         <is>
-          <t>재사용 금지 범위·초기화 기준·1:1 처리</t>
+          <t>방어 외 효과가 섞인 스킬도 전부 차단할지</t>
         </is>
       </c>
       <c r="G28" s="28" t="inlineStr">
@@ -5322,27 +5337,27 @@
       <c r="A29" s="51"/>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>도발과 복합 스킬</t>
+          <t>포자 발동 기준</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>방어스킬을 전부 제한한다는 사용자 편집을 유지한다.</t>
+          <t>스택이 쌓이고 발동 시 피해+암실. 3턴·3겹 기준은 추후 판단한다.</t>
         </is>
       </c>
       <c r="D29" s="1" t="inlineStr">
         <is>
-          <t>방어+공격·방어+다른 효과 스킬</t>
+          <t>기존: 다음 턴부터 1겹씩 증가, 3겹에서 발동·소모</t>
         </is>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>해로운 1턴 상태</t>
+          <t>조건부 상태</t>
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr">
         <is>
-          <t>방어 외 효과가 섞인 스킬도 전부 차단할지</t>
+          <t>3턴 경과와 3겹 도달 중 기준, 재부여·교체·발동 후 처리</t>
         </is>
       </c>
       <c r="G29" s="28" t="inlineStr">
@@ -5355,27 +5370,27 @@
       <c r="A30" s="51"/>
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>포자 발동 기준</t>
+          <t>포자 피해·암실 시점</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>스택이 쌓이고 발동 시 피해+암실. 3턴·3겹 기준은 추후 판단한다.</t>
+          <t>발동하면 피해와 1턴 암실을 함께 부여한다.</t>
         </is>
       </c>
       <c r="D30" s="1" t="inlineStr">
         <is>
-          <t>기존: 다음 턴부터 1겹씩 증가, 3겹에서 발동·소모</t>
+          <t>턴 끝 발동 후 자연 햇빛 처리</t>
         </is>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>조건부 상태</t>
+          <t>조건부→해로운 1턴 상태</t>
         </is>
       </c>
       <c r="F30" s="1" t="inlineStr">
         <is>
-          <t>3턴 경과와 3겹 도달 중 기준, 재부여·교체·발동 후 처리</t>
+          <t>피해량·피해 시점·암실의 적용 턴</t>
         </is>
       </c>
       <c r="G30" s="28" t="inlineStr">
@@ -5388,27 +5403,27 @@
       <c r="A31" s="51"/>
       <c r="B31" s="12" t="inlineStr">
         <is>
-          <t>포자 피해·암실 시점</t>
+          <t>그늘·암실 관계</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
-          <t>발동하면 피해와 1턴 암실을 함께 부여한다.</t>
+          <t>그늘은 환경으로 이동하고 암실은 개체의 1턴 상태로 둔다.</t>
         </is>
       </c>
       <c r="D31" s="1" t="inlineStr">
         <is>
-          <t>턴 끝 발동 후 자연 햇빛 처리</t>
+          <t>자연 햇빛 획득 방해</t>
         </is>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>조건부→해로운 1턴 상태</t>
+          <t>환경·해로운 1턴 상태</t>
         </is>
       </c>
       <c r="F31" s="1" t="inlineStr">
         <is>
-          <t>피해량·피해 시점·암실의 적용 턴</t>
+          <t>그늘의 적용 진영·지속 기준, 암실과 중복할 때 처리</t>
         </is>
       </c>
       <c r="G31" s="28" t="inlineStr">
@@ -5421,27 +5436,27 @@
       <c r="A32" s="51"/>
       <c r="B32" s="12" t="inlineStr">
         <is>
-          <t>그늘·암실 관계</t>
+          <t>갈증의 효과 연결</t>
         </is>
       </c>
       <c r="C32" s="12" t="inlineStr">
         <is>
-          <t>그늘은 환경으로 이동하고 암실은 개체의 1턴 상태로 둔다.</t>
+          <t>얘는 새로운 상태이상으로 만들지 말고 화상+암실 계속 갱신이 좋을 듯. 이름은 갈증으로</t>
         </is>
       </c>
       <c r="D32" s="1" t="inlineStr">
         <is>
-          <t>자연 햇빛 획득 방해</t>
+          <t>화상 해제 시 자연 해제 메모·기존 2턴</t>
         </is>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>환경·해로운 1턴 상태</t>
+          <t>스킬 부가 처리</t>
         </is>
       </c>
       <c r="F32" s="1" t="inlineStr">
         <is>
-          <t>그늘의 적용 진영·지속 기준, 암실과 중복할 때 처리</t>
+          <t>화상+암실 갱신 범위·종료 기준·지속</t>
         </is>
       </c>
       <c r="G32" s="28" t="inlineStr">
@@ -5454,12 +5469,12 @@
       <c r="A33" s="51"/>
       <c r="B33" s="12" t="inlineStr">
         <is>
-          <t>갈증의 효과 연결</t>
+          <t>지옥 불의 화상 중첩</t>
         </is>
       </c>
       <c r="C33" s="12" t="inlineStr">
         <is>
-          <t>얘는 새로운 상태이상으로 만들지 말고 화상+암실 계속 갱신이 좋을 듯. 이름은 갈증으로</t>
+          <t>얘도 새로운 상태이상이 아닌 화상의 중첩느낌으로 하자. 화상은 독처럼 중첩이 없었으나 이 스킬이 붙으면 중첩이 되는 ui로 바꾸는 걸로. 새로운 상태이상으로 취급하지는 말자.</t>
         </is>
       </c>
       <c r="D33" s="1" t="inlineStr">
@@ -5474,7 +5489,7 @@
       </c>
       <c r="F33" s="1" t="inlineStr">
         <is>
-          <t>화상+암실 갱신 범위·종료 기준·지속</t>
+          <t>중첩 수·상한·기간·재부여·표시 방식</t>
         </is>
       </c>
       <c r="G33" s="28" t="inlineStr">
@@ -5487,27 +5502,27 @@
       <c r="A34" s="51"/>
       <c r="B34" s="12" t="inlineStr">
         <is>
-          <t>지옥 불의 화상 중첩</t>
+          <t>기생·재생의 기간과 횟수</t>
         </is>
       </c>
       <c r="C34" s="12" t="inlineStr">
         <is>
-          <t>얘도 새로운 상태이상이 아닌 화상의 중첩느낌으로 하자. 화상은 독처럼 중첩이 없었으나 이 스킬이 붙으면 중첩이 되는 ui로 바꾸는 걸로. 새로운 상태이상으로 취급하지는 말자.</t>
+          <t>기간3은 턴마다 남은 기간을 줄이고, 횟수3은 실제 피해·회복이 발생한 횟수를 센다.</t>
         </is>
       </c>
       <c r="D34" s="1" t="inlineStr">
         <is>
-          <t>화상 해제 시 자연 해제 메모·기존 2턴</t>
+          <t>대기석·연결 끊김·발동 불가 시 차이</t>
         </is>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>스킬 부가 처리</t>
+          <t>기간 상태·공통 발동 규칙</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>중첩 수·상한·기간·재부여·표시 방식</t>
+          <t>현재는 기간3 유지. 대기·발동 불가 때도 감소할지</t>
         </is>
       </c>
       <c r="G34" s="28" t="inlineStr">
@@ -5520,63 +5535,30 @@
       <c r="A35" s="51"/>
       <c r="B35" s="12" t="inlineStr">
         <is>
-          <t>기생·재생의 기간과 횟수</t>
+          <t>봉인·속박의 불 해제</t>
         </is>
       </c>
       <c r="C35" s="12" t="inlineStr">
         <is>
-          <t>기간3은 턴마다 남은 기간을 줄이고, 횟수3은 실제 피해·회복이 발생한 횟수를 센다.</t>
+          <t>봉인은 기존 덩쿨의 새 이름이며 과거 불 피격 해제 조건은 재논의 중이다.</t>
         </is>
       </c>
       <c r="D35" s="1" t="inlineStr">
         <is>
-          <t>대기석·연결 끊김·발동 불가 시 차이</t>
+          <t>불타입 사용 제약도 함께 논의</t>
         </is>
       </c>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>기간 상태·공통 발동 규칙</t>
+          <t>해로운 1턴 상태</t>
         </is>
       </c>
       <c r="F35" s="1" t="inlineStr">
         <is>
-          <t>현재는 기간3 유지. 대기·발동 불가 때도 감소할지</t>
+          <t>불속성으로 해제할지와 적용 조건</t>
         </is>
       </c>
       <c r="G35" s="28" t="inlineStr">
-        <is>
-          <t>미결</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" spans="1:7" ht="100" customHeight="1">
-      <c r="A36" s="51"/>
-      <c r="B36" s="12" t="inlineStr">
-        <is>
-          <t>봉인·속박의 불 해제</t>
-        </is>
-      </c>
-      <c r="C36" s="12" t="inlineStr">
-        <is>
-          <t>봉인은 기존 덩쿨의 새 이름이며 과거 불 피격 해제 조건은 재논의 중이다.</t>
-        </is>
-      </c>
-      <c r="D36" s="1" t="inlineStr">
-        <is>
-          <t>불타입 사용 제약도 함께 논의</t>
-        </is>
-      </c>
-      <c r="E36" s="1" t="inlineStr">
-        <is>
-          <t>해로운 1턴 상태</t>
-        </is>
-      </c>
-      <c r="F36" s="1" t="inlineStr">
-        <is>
-          <t>불속성으로 해제할지와 적용 조건</t>
-        </is>
-      </c>
-      <c r="G36" s="28" t="inlineStr">
         <is>
           <t>미결</t>
         </is>
@@ -5585,14 +5567,14 @@
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A6:A12"/>
-    <mergeCell ref="A13:A16"/>
-    <mergeCell ref="A17:A24"/>
-    <mergeCell ref="A25:A36"/>
+    <mergeCell ref="A6:A11"/>
+    <mergeCell ref="A12:A15"/>
+    <mergeCell ref="A16:A23"/>
+    <mergeCell ref="A24:A35"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="G6:G24" xr:uid="{00000000-0002-0000-0200-000000000000}">
+    <dataValidation type="list" sqref="G6:G23" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"보류,유지,통합,삭제"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5817,4 +5799,135 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <sheetPr>
+    <tabColor rgb="FFB58B37"/>
+  </sheetPr>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr defaultRowHeight="14"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="23" customWidth="1"/>
+    <col min="3" max="3" width="59" customWidth="1"/>
+    <col min="4" max="4" width="51" customWidth="1"/>
+    <col min="5" max="5" width="31" customWidth="1"/>
+    <col min="6" max="6" width="55" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="17">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="2" spans="1:7" ht="30" customHeight="1">
+      <c r="A2" s="57" t="inlineStr">
+        <is>
+          <t>보류한 처리와 스킬</t>
+        </is>
+      </c>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+    </row>
+    <row r="3" spans="1:7" ht="17">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+    </row>
+    <row r="4" spans="1:7" ht="17">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+    </row>
+    <row r="5" spans="1:7" ht="30" customHeight="1">
+      <c r="A5" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="42" customHeight="1">
+      <c r="A6" s="47" t="inlineStr">
+        <is>
+          <t>처리 용어</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>모으기</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>이번 행동에 준비하고 다음 행동에 예약된 공격을 실행하는 기존 공통 장치다.</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>공통 장치의 2단계 공격 예약. 현재 은신 통합 규칙과는 별개</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>공격 스킬 후보</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>확정 고유스킬에 필요할 때 재검토</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="inlineStr">
+        <is>
+          <t>보류</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:G2"/>
+  </mergeCells>
+  <phoneticPr fontId="6" type="noConversion"/>
+  <dataValidations count="1">
+    <dataValidation type="list" sqref="G6" xr:uid="{00000000-0002-0000-0200-000000000000}">
+      <formula1>"보류,유지,통합,삭제"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>